<commit_message>
Correct biomarker flags and analysis ID coercion
</commit_message>
<xml_diff>
--- a/public/downloads/extended-reanalysis.xlsx
+++ b/public/downloads/extended-reanalysis.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R08c861dcbe2a4251"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key Findings" sheetId="2" r:id="Rb1935d533de14687"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benefit-Harm" sheetId="3" r:id="Ra2aeb3dcf57a4180"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent Results" sheetId="4" r:id="R279fe22f76544d49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Agent MD" sheetId="5" r:id="R215b79b32b094e0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Absolute Safety" sheetId="6" r:id="R19d64916fdd34ca3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Termination Sensitivity" sheetId="7" r:id="Rf84bf61dc9e241a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MID Compatibility" sheetId="8" r:id="Rdaea8a9169da4e24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Target Classes" sheetId="9" r:id="R2a5970b744024fba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interaction Tests" sheetId="10" r:id="Rbaea5ece55a74980"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Moderator Models" sheetId="11" r:id="Rf46ea4b50b2145e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leave-One-Out" sheetId="12" r:id="R1cb6f2a6d40b4a21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trial Annotations" sheetId="13" r:id="R14d868d59afc4321"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality Control" sheetId="14" r:id="R5d0a9397896d4678"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="R172f4f998e644cd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R0015f2f4e46948d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key Findings" sheetId="2" r:id="Rff259744d92c430b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benefit-Harm" sheetId="3" r:id="R3d09c2cfcee64c94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent Results" sheetId="4" r:id="Rcca4aff4109b4f86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Agent MD" sheetId="5" r:id="R81eebbf0dad74d49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Absolute Safety" sheetId="6" r:id="Rd38dbde858ab4b5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Termination Sensitivity" sheetId="7" r:id="R72e013d521544c4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MID Compatibility" sheetId="8" r:id="R3f392b9b580245cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Target Classes" sheetId="9" r:id="R0bb0dce58bc84bb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interaction Tests" sheetId="10" r:id="Rd310b0f6c85f4a91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Moderator Models" sheetId="11" r:id="Ra62f0df8e8304ca3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leave-One-Out" sheetId="12" r:id="Ree37007389bd4315"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trial Annotations" sheetId="13" r:id="Ra51c4250a5054608"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality Control" sheetId="14" r:id="R246dfa8d847644f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="R672c0f5fa49d44af"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -522,7 +522,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R65ec3e68b04449d5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R10d08953f0214bb2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -639,7 +639,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="TerminationTable" displayName="TerminationTable" ref="A4:J99" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="TerminationTable" displayName="TerminationTable" ref="A4:J102" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Outcome"/>
@@ -1531,7 +1531,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38213bf862054799"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9ec5947e1d047e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2049,7 +2049,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R848e47379e804e18"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R410565805a7b4fc8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3429,7 +3429,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85b7a3a2242741a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62f1d308bfed448b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3790,10 +3790,10 @@
         <x:v>Futility</x:v>
       </x:c>
       <x:c r="G16" s="50" t="str">
-        <x:v>Not uniformly required</x:v>
+        <x:v>Required</x:v>
       </x:c>
       <x:c r="H16" s="50" t="str">
-        <x:v>Cochrane CD016297 ref 100</x:v>
+        <x:v>Cochrane CD016297 ref 100 and study description</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -3816,10 +3816,10 @@
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="G17" s="50" t="str">
-        <x:v>Not uniformly required</x:v>
+        <x:v>Required</x:v>
       </x:c>
       <x:c r="H17" s="50" t="str">
-        <x:v>Cochrane CD016297 refs 96/110</x:v>
+        <x:v>Cochrane CD016297 refs 96/110 and study description</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -3842,10 +3842,10 @@
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="G18" s="50" t="str">
-        <x:v>Not uniformly required</x:v>
+        <x:v>Required</x:v>
       </x:c>
       <x:c r="H18" s="50" t="str">
-        <x:v>Cochrane CD016297 refs 96/110</x:v>
+        <x:v>Cochrane CD016297 refs 96/110 and study description</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -3933,7 +3933,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R976dd50de23a4db1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b96807deef8409a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4351,7 +4351,7 @@
     <x:mergeCell ref="A36:L36"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b98d20a32d84567"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab68701b47a846b1"/>
 </x:worksheet>
 </file>
 
@@ -4509,7 +4509,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2c235a303c34aef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd0ff9fe2c994658"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6078,7 +6078,7 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="50" t="str">
-        <x:v>4.1</x:v>
+        <x:v>4.10</x:v>
       </x:c>
       <x:c r="B50" s="50" t="str">
         <x:v>Symptomatic ARIA H at 18 months</x:v>
@@ -7925,7 +7925,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d8092fe9f2a4e17"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60f4b569eba14d92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8771,7 +8771,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41ad6afae1184a06"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e26071aa7bd43ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8946,7 +8946,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="50" t="str">
-        <x:v>4.1</x:v>
+        <x:v>4.10</x:v>
       </x:c>
       <x:c r="B7" s="50" t="str">
         <x:v>Symptomatic ARIA H at 18 months</x:v>
@@ -11442,7 +11442,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9221f5a79aa4482d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75f4afb8b5fa42d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12789,19 +12789,19 @@
         <x:v>Cochrane class pool</x:v>
       </x:c>
       <x:c r="E45" s="59" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F45" s="62" t="n">
-        <x:v>2.401027274738645</x:v>
+        <x:v>2.396697026053298</x:v>
       </x:c>
       <x:c r="G45" s="62" t="n">
-        <x:v>2.084713423767042</x:v>
+        <x:v>2.074870925771338</x:v>
       </x:c>
       <x:c r="H45" s="62" t="n">
-        <x:v>2.76533546928563</x:v>
+        <x:v>2.768440466993058</x:v>
       </x:c>
       <x:c r="I45" s="65" t="n">
-        <x:v>0.001402098015329501</x:v>
+        <x:v>1.481404164582036e-32</x:v>
       </x:c>
       <x:c r="J45" s="56" t="n">
         <x:v>0</x:v>
@@ -12821,19 +12821,19 @@
         <x:v>Exclude futility-terminated trials</x:v>
       </x:c>
       <x:c r="E46" s="59" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F46" s="62" t="n">
-        <x:v>2.401027274738645</x:v>
+        <x:v>2.396697026053298</x:v>
       </x:c>
       <x:c r="G46" s="62" t="n">
-        <x:v>2.084713423767042</x:v>
+        <x:v>2.074870925771338</x:v>
       </x:c>
       <x:c r="H46" s="62" t="n">
-        <x:v>2.76533546928563</x:v>
+        <x:v>2.768440466993058</x:v>
       </x:c>
       <x:c r="I46" s="65" t="n">
-        <x:v>0.001402098015329501</x:v>
+        <x:v>1.481404164582036e-32</x:v>
       </x:c>
       <x:c r="J46" s="56" t="n">
         <x:v>0</x:v>
@@ -12853,19 +12853,19 @@
         <x:v>Exclude all early-terminated trials</x:v>
       </x:c>
       <x:c r="E47" s="59" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F47" s="62" t="n">
-        <x:v>2.401027274738645</x:v>
+        <x:v>2.396697026053298</x:v>
       </x:c>
       <x:c r="G47" s="62" t="n">
-        <x:v>2.084713423767042</x:v>
+        <x:v>2.074870925771338</x:v>
       </x:c>
       <x:c r="H47" s="62" t="n">
-        <x:v>2.76533546928563</x:v>
+        <x:v>2.768440466993058</x:v>
       </x:c>
       <x:c r="I47" s="65" t="n">
-        <x:v>0.001402098015329501</x:v>
+        <x:v>1.481404164582036e-32</x:v>
       </x:c>
       <x:c r="J47" s="56" t="n">
         <x:v>0</x:v>
@@ -13573,10 +13573,10 @@
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="50" t="str">
-        <x:v>5.1</x:v>
+        <x:v>4.10</x:v>
       </x:c>
       <x:c r="B70" s="50" t="str">
-        <x:v>SAE at 18 months</x:v>
+        <x:v>Symptomatic ARIA H at 18 months</x:v>
       </x:c>
       <x:c r="C70" s="50" t="str">
         <x:v>RR</x:v>
@@ -13585,30 +13585,28 @@
         <x:v>Cochrane class pool</x:v>
       </x:c>
       <x:c r="E70" s="59" t="n">
-        <x:v>9</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F70" s="62" t="n">
-        <x:v>1.041125919875473</x:v>
+        <x:v>2.996659242761694</x:v>
       </x:c>
       <x:c r="G70" s="62" t="n">
-        <x:v>0.9197385260982464</x:v>
+        <x:v>0.6064524420319731</x:v>
       </x:c>
       <x:c r="H70" s="62" t="n">
-        <x:v>1.178534061887023</x:v>
+        <x:v>14.807371518104377</x:v>
       </x:c>
       <x:c r="I70" s="65" t="n">
-        <x:v>0.4749065574334277</x:v>
-      </x:c>
-      <x:c r="J70" s="56" t="n">
-        <x:v>39.37245648976637</x:v>
-      </x:c>
+        <x:v>0.1781711995829671</x:v>
+      </x:c>
+      <x:c r="J70" s="56"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="50" t="str">
-        <x:v>5.1</x:v>
+        <x:v>4.10</x:v>
       </x:c>
       <x:c r="B71" s="50" t="str">
-        <x:v>SAE at 18 months</x:v>
+        <x:v>Symptomatic ARIA H at 18 months</x:v>
       </x:c>
       <x:c r="C71" s="50" t="str">
         <x:v>RR</x:v>
@@ -13617,30 +13615,28 @@
         <x:v>Exclude futility-terminated trials</x:v>
       </x:c>
       <x:c r="E71" s="59" t="n">
-        <x:v>6</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F71" s="62" t="n">
-        <x:v>1.083436096979602</x:v>
+        <x:v>2.996659242761694</x:v>
       </x:c>
       <x:c r="G71" s="62" t="n">
-        <x:v>0.9197977450241073</x:v>
+        <x:v>0.6064524420319731</x:v>
       </x:c>
       <x:c r="H71" s="62" t="n">
-        <x:v>1.276186838452869</x:v>
+        <x:v>14.807371518104377</x:v>
       </x:c>
       <x:c r="I71" s="65" t="n">
-        <x:v>0.2639087413676368</x:v>
-      </x:c>
-      <x:c r="J71" s="56" t="n">
-        <x:v>50.76790651647276</x:v>
-      </x:c>
+        <x:v>0.1781711995829671</x:v>
+      </x:c>
+      <x:c r="J71" s="56"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="50" t="str">
-        <x:v>5.1</x:v>
+        <x:v>4.10</x:v>
       </x:c>
       <x:c r="B72" s="50" t="str">
-        <x:v>SAE at 18 months</x:v>
+        <x:v>Symptomatic ARIA H at 18 months</x:v>
       </x:c>
       <x:c r="C72" s="50" t="str">
         <x:v>RR</x:v>
@@ -13649,30 +13645,28 @@
         <x:v>Exclude all early-terminated trials</x:v>
       </x:c>
       <x:c r="E72" s="59" t="n">
-        <x:v>6</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F72" s="62" t="n">
-        <x:v>1.083436096979602</x:v>
+        <x:v>2.996659242761694</x:v>
       </x:c>
       <x:c r="G72" s="62" t="n">
-        <x:v>0.9197977450241073</x:v>
+        <x:v>0.6064524420319731</x:v>
       </x:c>
       <x:c r="H72" s="62" t="n">
-        <x:v>1.276186838452869</x:v>
+        <x:v>14.807371518104377</x:v>
       </x:c>
       <x:c r="I72" s="65" t="n">
-        <x:v>0.2639087413676368</x:v>
-      </x:c>
-      <x:c r="J72" s="56" t="n">
-        <x:v>50.76790651647276</x:v>
-      </x:c>
+        <x:v>0.1781711995829671</x:v>
+      </x:c>
+      <x:c r="J72" s="56"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="50" t="str">
-        <x:v>5.2</x:v>
+        <x:v>5.1</x:v>
       </x:c>
       <x:c r="B73" s="50" t="str">
-        <x:v>SAE at 24 months</x:v>
+        <x:v>SAE at 18 months</x:v>
       </x:c>
       <x:c r="C73" s="50" t="str">
         <x:v>RR</x:v>
@@ -13681,30 +13675,30 @@
         <x:v>Cochrane class pool</x:v>
       </x:c>
       <x:c r="E73" s="59" t="n">
-        <x:v>4</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="F73" s="62" t="n">
-        <x:v>1.03100110180081</x:v>
+        <x:v>1.041125919875473</x:v>
       </x:c>
       <x:c r="G73" s="62" t="n">
-        <x:v>0.7922103769561634</x:v>
+        <x:v>0.9197385260982464</x:v>
       </x:c>
       <x:c r="H73" s="62" t="n">
-        <x:v>1.341768932639596</x:v>
+        <x:v>1.178534061887023</x:v>
       </x:c>
       <x:c r="I73" s="65" t="n">
-        <x:v>0.7367734785731431</x:v>
+        <x:v>0.4749065574334277</x:v>
       </x:c>
       <x:c r="J73" s="56" t="n">
-        <x:v>0</x:v>
+        <x:v>39.37245648976637</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="50" t="str">
-        <x:v>5.2</x:v>
+        <x:v>5.1</x:v>
       </x:c>
       <x:c r="B74" s="50" t="str">
-        <x:v>SAE at 24 months</x:v>
+        <x:v>SAE at 18 months</x:v>
       </x:c>
       <x:c r="C74" s="50" t="str">
         <x:v>RR</x:v>
@@ -13713,81 +13707,83 @@
         <x:v>Exclude futility-terminated trials</x:v>
       </x:c>
       <x:c r="E74" s="59" t="n">
-        <x:v>1</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F74" s="62" t="n">
-        <x:v>1.29769820971867</x:v>
+        <x:v>1.083436096979602</x:v>
       </x:c>
       <x:c r="G74" s="62" t="n">
-        <x:v>0.8159302297730878</x:v>
+        <x:v>0.9197977450241073</x:v>
       </x:c>
       <x:c r="H74" s="62" t="n">
-        <x:v>2.063927260024882</x:v>
+        <x:v>1.276186838452869</x:v>
       </x:c>
       <x:c r="I74" s="65" t="n">
-        <x:v>0.2710216887898833</x:v>
-      </x:c>
-      <x:c r="J74" s="56"/>
+        <x:v>0.2639087413676368</x:v>
+      </x:c>
+      <x:c r="J74" s="56" t="n">
+        <x:v>50.76790651647276</x:v>
+      </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="50" t="str">
-        <x:v>5.3</x:v>
+        <x:v>5.1</x:v>
       </x:c>
       <x:c r="B75" s="50" t="str">
-        <x:v>SAE above 24 months</x:v>
+        <x:v>SAE at 18 months</x:v>
       </x:c>
       <x:c r="C75" s="50" t="str">
         <x:v>RR</x:v>
       </x:c>
       <x:c r="D75" s="50" t="str">
-        <x:v>Cochrane class pool</x:v>
+        <x:v>Exclude all early-terminated trials</x:v>
       </x:c>
       <x:c r="E75" s="59" t="n">
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F75" s="62" t="n">
-        <x:v>0.8237606397871372</x:v>
+        <x:v>1.083436096979602</x:v>
       </x:c>
       <x:c r="G75" s="62" t="n">
-        <x:v>0.6672245404164605</x:v>
+        <x:v>0.9197977450241073</x:v>
       </x:c>
       <x:c r="H75" s="62" t="n">
-        <x:v>1.017021333236581</x:v>
+        <x:v>1.276186838452869</x:v>
       </x:c>
       <x:c r="I75" s="65" t="n">
-        <x:v>0.0713880407286846</x:v>
+        <x:v>0.2639087413676368</x:v>
       </x:c>
       <x:c r="J75" s="56" t="n">
-        <x:v>0</x:v>
+        <x:v>50.76790651647276</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="50" t="str">
-        <x:v>5.3</x:v>
+        <x:v>5.2</x:v>
       </x:c>
       <x:c r="B76" s="50" t="str">
-        <x:v>SAE above 24 months</x:v>
+        <x:v>SAE at 24 months</x:v>
       </x:c>
       <x:c r="C76" s="50" t="str">
         <x:v>RR</x:v>
       </x:c>
       <x:c r="D76" s="50" t="str">
-        <x:v>Exclude futility-terminated trials</x:v>
+        <x:v>Cochrane class pool</x:v>
       </x:c>
       <x:c r="E76" s="59" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F76" s="62" t="n">
-        <x:v>0.8237606397871372</x:v>
+        <x:v>1.03100110180081</x:v>
       </x:c>
       <x:c r="G76" s="62" t="n">
-        <x:v>0.6672245404164605</x:v>
+        <x:v>0.7922103769561634</x:v>
       </x:c>
       <x:c r="H76" s="62" t="n">
-        <x:v>1.017021333236581</x:v>
+        <x:v>1.341768932639596</x:v>
       </x:c>
       <x:c r="I76" s="65" t="n">
-        <x:v>0.0713880407286846</x:v>
+        <x:v>0.7367734785731431</x:v>
       </x:c>
       <x:c r="J76" s="56" t="n">
         <x:v>0</x:v>
@@ -13795,42 +13791,40 @@
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="50" t="str">
-        <x:v>5.3</x:v>
+        <x:v>5.2</x:v>
       </x:c>
       <x:c r="B77" s="50" t="str">
-        <x:v>SAE above 24 months</x:v>
+        <x:v>SAE at 24 months</x:v>
       </x:c>
       <x:c r="C77" s="50" t="str">
         <x:v>RR</x:v>
       </x:c>
       <x:c r="D77" s="50" t="str">
-        <x:v>Exclude all early-terminated trials</x:v>
+        <x:v>Exclude futility-terminated trials</x:v>
       </x:c>
       <x:c r="E77" s="59" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F77" s="62" t="n">
-        <x:v>0.8237606397871372</x:v>
+        <x:v>1.29769820971867</x:v>
       </x:c>
       <x:c r="G77" s="62" t="n">
-        <x:v>0.6672245404164605</x:v>
+        <x:v>0.8159302297730878</x:v>
       </x:c>
       <x:c r="H77" s="62" t="n">
-        <x:v>1.017021333236581</x:v>
+        <x:v>2.063927260024882</x:v>
       </x:c>
       <x:c r="I77" s="65" t="n">
-        <x:v>0.0713880407286846</x:v>
-      </x:c>
-      <x:c r="J77" s="56" t="n">
-        <x:v>0</x:v>
-      </x:c>
+        <x:v>0.2710216887898833</x:v>
+      </x:c>
+      <x:c r="J77" s="56"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="50" t="str">
-        <x:v>6.1</x:v>
+        <x:v>5.3</x:v>
       </x:c>
       <x:c r="B78" s="50" t="str">
-        <x:v>Mortality at 18 months</x:v>
+        <x:v>SAE above 24 months</x:v>
       </x:c>
       <x:c r="C78" s="50" t="str">
         <x:v>RR</x:v>
@@ -13839,30 +13833,30 @@
         <x:v>Cochrane class pool</x:v>
       </x:c>
       <x:c r="E78" s="59" t="n">
-        <x:v>7</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F78" s="62" t="n">
-        <x:v>1.172699932526192</x:v>
+        <x:v>0.8237606397871372</x:v>
       </x:c>
       <x:c r="G78" s="62" t="n">
-        <x:v>0.6151622791578121</x:v>
+        <x:v>0.6672245404164605</x:v>
       </x:c>
       <x:c r="H78" s="62" t="n">
-        <x:v>2.235548534656072</x:v>
+        <x:v>1.017021333236581</x:v>
       </x:c>
       <x:c r="I78" s="65" t="n">
-        <x:v>0.5678400901058178</x:v>
+        <x:v>0.0713880407286846</x:v>
       </x:c>
       <x:c r="J78" s="56" t="n">
-        <x:v>31.573527502497875</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="50" t="str">
-        <x:v>6.1</x:v>
+        <x:v>5.3</x:v>
       </x:c>
       <x:c r="B79" s="50" t="str">
-        <x:v>Mortality at 18 months</x:v>
+        <x:v>SAE above 24 months</x:v>
       </x:c>
       <x:c r="C79" s="50" t="str">
         <x:v>RR</x:v>
@@ -13871,30 +13865,30 @@
         <x:v>Exclude futility-terminated trials</x:v>
       </x:c>
       <x:c r="E79" s="59" t="n">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F79" s="62" t="n">
-        <x:v>1.253703494367707</x:v>
+        <x:v>0.8237606397871372</x:v>
       </x:c>
       <x:c r="G79" s="62" t="n">
-        <x:v>0.7155400652075709</x:v>
+        <x:v>0.6672245404164605</x:v>
       </x:c>
       <x:c r="H79" s="62" t="n">
-        <x:v>2.196623960300316</x:v>
+        <x:v>1.017021333236581</x:v>
       </x:c>
       <x:c r="I79" s="65" t="n">
-        <x:v>0.3475296231744265</x:v>
+        <x:v>0.0713880407286846</x:v>
       </x:c>
       <x:c r="J79" s="56" t="n">
-        <x:v>30.824015654990806</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="50" t="str">
-        <x:v>6.1</x:v>
+        <x:v>5.3</x:v>
       </x:c>
       <x:c r="B80" s="50" t="str">
-        <x:v>Mortality at 18 months</x:v>
+        <x:v>SAE above 24 months</x:v>
       </x:c>
       <x:c r="C80" s="50" t="str">
         <x:v>RR</x:v>
@@ -13903,30 +13897,30 @@
         <x:v>Exclude all early-terminated trials</x:v>
       </x:c>
       <x:c r="E80" s="59" t="n">
-        <x:v>6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F80" s="62" t="n">
-        <x:v>1.253703494367707</x:v>
+        <x:v>0.8237606397871372</x:v>
       </x:c>
       <x:c r="G80" s="62" t="n">
-        <x:v>0.7155400652075709</x:v>
+        <x:v>0.6672245404164605</x:v>
       </x:c>
       <x:c r="H80" s="62" t="n">
-        <x:v>2.196623960300316</x:v>
+        <x:v>1.017021333236581</x:v>
       </x:c>
       <x:c r="I80" s="65" t="n">
-        <x:v>0.3475296231744265</x:v>
+        <x:v>0.0713880407286846</x:v>
       </x:c>
       <x:c r="J80" s="56" t="n">
-        <x:v>30.824015654990806</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="50" t="str">
-        <x:v>6.2</x:v>
+        <x:v>6.1</x:v>
       </x:c>
       <x:c r="B81" s="50" t="str">
-        <x:v>Mortality at 24 months</x:v>
+        <x:v>Mortality at 18 months</x:v>
       </x:c>
       <x:c r="C81" s="50" t="str">
         <x:v>RR</x:v>
@@ -13935,30 +13929,30 @@
         <x:v>Cochrane class pool</x:v>
       </x:c>
       <x:c r="E81" s="59" t="n">
-        <x:v>4</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F81" s="62" t="n">
-        <x:v>1.054613984226481</x:v>
+        <x:v>1.172699932526192</x:v>
       </x:c>
       <x:c r="G81" s="62" t="n">
-        <x:v>0.2914924045683833</x:v>
+        <x:v>0.6151622791578121</x:v>
       </x:c>
       <x:c r="H81" s="62" t="n">
-        <x:v>3.815573367590551</x:v>
+        <x:v>2.235548534656072</x:v>
       </x:c>
       <x:c r="I81" s="65" t="n">
-        <x:v>0.9036308770545904</x:v>
+        <x:v>0.5678400901058178</x:v>
       </x:c>
       <x:c r="J81" s="56" t="n">
-        <x:v>7.878428238569578</x:v>
+        <x:v>31.573527502497875</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="50" t="str">
-        <x:v>6.2</x:v>
+        <x:v>6.1</x:v>
       </x:c>
       <x:c r="B82" s="50" t="str">
-        <x:v>Mortality at 24 months</x:v>
+        <x:v>Mortality at 18 months</x:v>
       </x:c>
       <x:c r="C82" s="50" t="str">
         <x:v>RR</x:v>
@@ -13967,312 +13961,312 @@
         <x:v>Exclude futility-terminated trials</x:v>
       </x:c>
       <x:c r="E82" s="59" t="n">
-        <x:v>1</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F82" s="62" t="n">
-        <x:v>3.546255506607929</x:v>
+        <x:v>1.253703494367707</x:v>
       </x:c>
       <x:c r="G82" s="62" t="n">
-        <x:v>0.1836978958395782</x:v>
+        <x:v>0.7155400652075709</x:v>
       </x:c>
       <x:c r="H82" s="62" t="n">
-        <x:v>68.45983760820818</x:v>
+        <x:v>2.196623960300316</x:v>
       </x:c>
       <x:c r="I82" s="65" t="n">
-        <x:v>0.4019689066760839</x:v>
-      </x:c>
-      <x:c r="J82" s="56"/>
+        <x:v>0.3475296231744265</x:v>
+      </x:c>
+      <x:c r="J82" s="56" t="n">
+        <x:v>30.824015654990806</x:v>
+      </x:c>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="50" t="str">
-        <x:v>6.3</x:v>
+        <x:v>6.1</x:v>
       </x:c>
       <x:c r="B83" s="50" t="str">
-        <x:v>Mortality above 24 months</x:v>
+        <x:v>Mortality at 18 months</x:v>
       </x:c>
       <x:c r="C83" s="50" t="str">
         <x:v>RR</x:v>
       </x:c>
       <x:c r="D83" s="50" t="str">
-        <x:v>Cochrane class pool</x:v>
+        <x:v>Exclude all early-terminated trials</x:v>
       </x:c>
       <x:c r="E83" s="59" t="n">
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F83" s="62" t="n">
-        <x:v>0.6972000337432346</x:v>
+        <x:v>1.253703494367707</x:v>
       </x:c>
       <x:c r="G83" s="62" t="n">
-        <x:v>0.1251357066798499</x:v>
+        <x:v>0.7155400652075709</x:v>
       </x:c>
       <x:c r="H83" s="62" t="n">
-        <x:v>3.884485890947067</x:v>
+        <x:v>2.196623960300316</x:v>
       </x:c>
       <x:c r="I83" s="65" t="n">
-        <x:v>0.6806620419187537</x:v>
+        <x:v>0.3475296231744265</x:v>
       </x:c>
       <x:c r="J83" s="56" t="n">
-        <x:v>73.3779120362122</x:v>
+        <x:v>30.824015654990806</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="50" t="str">
-        <x:v>6.3</x:v>
+        <x:v>6.2</x:v>
       </x:c>
       <x:c r="B84" s="50" t="str">
-        <x:v>Mortality above 24 months</x:v>
+        <x:v>Mortality at 24 months</x:v>
       </x:c>
       <x:c r="C84" s="50" t="str">
         <x:v>RR</x:v>
       </x:c>
       <x:c r="D84" s="50" t="str">
-        <x:v>Exclude futility-terminated trials</x:v>
+        <x:v>Cochrane class pool</x:v>
       </x:c>
       <x:c r="E84" s="59" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F84" s="62" t="n">
-        <x:v>0.6972000337432346</x:v>
+        <x:v>1.054613984226481</x:v>
       </x:c>
       <x:c r="G84" s="62" t="n">
-        <x:v>0.1251357066798499</x:v>
+        <x:v>0.2914924045683833</x:v>
       </x:c>
       <x:c r="H84" s="62" t="n">
-        <x:v>3.884485890947067</x:v>
+        <x:v>3.815573367590551</x:v>
       </x:c>
       <x:c r="I84" s="65" t="n">
-        <x:v>0.6806620419187537</x:v>
+        <x:v>0.9036308770545904</x:v>
       </x:c>
       <x:c r="J84" s="56" t="n">
-        <x:v>73.3779120362122</x:v>
+        <x:v>7.878428238569578</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="50" t="str">
-        <x:v>6.3</x:v>
+        <x:v>6.2</x:v>
       </x:c>
       <x:c r="B85" s="50" t="str">
-        <x:v>Mortality above 24 months</x:v>
+        <x:v>Mortality at 24 months</x:v>
       </x:c>
       <x:c r="C85" s="50" t="str">
         <x:v>RR</x:v>
       </x:c>
       <x:c r="D85" s="50" t="str">
-        <x:v>Exclude all early-terminated trials</x:v>
+        <x:v>Exclude futility-terminated trials</x:v>
       </x:c>
       <x:c r="E85" s="59" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F85" s="62" t="n">
-        <x:v>0.6972000337432346</x:v>
+        <x:v>3.546255506607929</x:v>
       </x:c>
       <x:c r="G85" s="62" t="n">
-        <x:v>0.1251357066798499</x:v>
+        <x:v>0.1836978958395782</x:v>
       </x:c>
       <x:c r="H85" s="62" t="n">
-        <x:v>3.884485890947067</x:v>
+        <x:v>68.45983760820818</x:v>
       </x:c>
       <x:c r="I85" s="65" t="n">
-        <x:v>0.6806620419187537</x:v>
-      </x:c>
-      <x:c r="J85" s="56" t="n">
-        <x:v>73.3779120362122</x:v>
-      </x:c>
+        <x:v>0.4019689066760839</x:v>
+      </x:c>
+      <x:c r="J85" s="56"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="50" t="str">
-        <x:v>7.1</x:v>
+        <x:v>6.3</x:v>
       </x:c>
       <x:c r="B86" s="50" t="str">
-        <x:v>NPI-Q score at 12 months</x:v>
+        <x:v>Mortality above 24 months</x:v>
       </x:c>
       <x:c r="C86" s="50" t="str">
-        <x:v>SMD</x:v>
+        <x:v>RR</x:v>
       </x:c>
       <x:c r="D86" s="50" t="str">
         <x:v>Cochrane class pool</x:v>
       </x:c>
       <x:c r="E86" s="59" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F86" s="62" t="n">
-        <x:v>0.08604846600191733</x:v>
+        <x:v>0.6972000337432346</x:v>
       </x:c>
       <x:c r="G86" s="62" t="n">
-        <x:v>-0.1834920094196857</x:v>
+        <x:v>0.1251357066798499</x:v>
       </x:c>
       <x:c r="H86" s="62" t="n">
-        <x:v>0.3555889414235204</x:v>
+        <x:v>3.884485890947067</x:v>
       </x:c>
       <x:c r="I86" s="65" t="n">
-        <x:v>0.5315107139042438</x:v>
-      </x:c>
-      <x:c r="J86" s="56"/>
+        <x:v>0.6806620419187537</x:v>
+      </x:c>
+      <x:c r="J86" s="56" t="n">
+        <x:v>73.3779120362122</x:v>
+      </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="50" t="str">
-        <x:v>7.2</x:v>
+        <x:v>6.3</x:v>
       </x:c>
       <x:c r="B87" s="50" t="str">
-        <x:v>NPI-Q score at 18 months</x:v>
+        <x:v>Mortality above 24 months</x:v>
       </x:c>
       <x:c r="C87" s="50" t="str">
-        <x:v>SMD</x:v>
+        <x:v>RR</x:v>
       </x:c>
       <x:c r="D87" s="50" t="str">
-        <x:v>Cochrane class pool</x:v>
+        <x:v>Exclude futility-terminated trials</x:v>
       </x:c>
       <x:c r="E87" s="59" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F87" s="62" t="n">
-        <x:v>0.1191993997701558</x:v>
+        <x:v>0.6972000337432346</x:v>
       </x:c>
       <x:c r="G87" s="62" t="n">
-        <x:v>-0.1747924558477071</x:v>
+        <x:v>0.1251357066798499</x:v>
       </x:c>
       <x:c r="H87" s="62" t="n">
-        <x:v>0.4131912553880188</x:v>
+        <x:v>3.884485890947067</x:v>
       </x:c>
       <x:c r="I87" s="65" t="n">
-        <x:v>0.4268054428964087</x:v>
+        <x:v>0.6806620419187537</x:v>
       </x:c>
       <x:c r="J87" s="56" t="n">
-        <x:v>0</x:v>
+        <x:v>73.3779120362122</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="50" t="str">
-        <x:v>7.2</x:v>
+        <x:v>6.3</x:v>
       </x:c>
       <x:c r="B88" s="50" t="str">
-        <x:v>NPI-Q score at 18 months</x:v>
+        <x:v>Mortality above 24 months</x:v>
       </x:c>
       <x:c r="C88" s="50" t="str">
-        <x:v>SMD</x:v>
+        <x:v>RR</x:v>
       </x:c>
       <x:c r="D88" s="50" t="str">
-        <x:v>Exclude futility-terminated trials</x:v>
+        <x:v>Exclude all early-terminated trials</x:v>
       </x:c>
       <x:c r="E88" s="59" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F88" s="62" t="n">
-        <x:v>0.5168562568898105</x:v>
+        <x:v>0.6972000337432346</x:v>
       </x:c>
       <x:c r="G88" s="62" t="n">
-        <x:v>-0.9579855762756353</x:v>
+        <x:v>0.1251357066798499</x:v>
       </x:c>
       <x:c r="H88" s="62" t="n">
-        <x:v>1.991698090055256</x:v>
+        <x:v>3.884485890947067</x:v>
       </x:c>
       <x:c r="I88" s="65" t="n">
-        <x:v>0.4921667733628572</x:v>
-      </x:c>
-      <x:c r="J88" s="56"/>
+        <x:v>0.6806620419187537</x:v>
+      </x:c>
+      <x:c r="J88" s="56" t="n">
+        <x:v>73.3779120362122</x:v>
+      </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="50" t="str">
-        <x:v>8.1</x:v>
+        <x:v>7.1</x:v>
       </x:c>
       <x:c r="B89" s="50" t="str">
-        <x:v>Infusion reaction at 18 months</x:v>
+        <x:v>NPI-Q score at 12 months</x:v>
       </x:c>
       <x:c r="C89" s="50" t="str">
-        <x:v>RR</x:v>
+        <x:v>SMD</x:v>
       </x:c>
       <x:c r="D89" s="50" t="str">
         <x:v>Cochrane class pool</x:v>
       </x:c>
       <x:c r="E89" s="59" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F89" s="62" t="n">
-        <x:v>3.580414000675479</x:v>
+        <x:v>0.08604846600191733</x:v>
       </x:c>
       <x:c r="G89" s="62" t="n">
-        <x:v>0.06906491805724485</x:v>
+        <x:v>-0.1834920094196857</x:v>
       </x:c>
       <x:c r="H89" s="62" t="n">
-        <x:v>185.61325745159925</x:v>
+        <x:v>0.3555889414235204</x:v>
       </x:c>
       <x:c r="I89" s="65" t="n">
-        <x:v>0.2990275366168896</x:v>
-      </x:c>
-      <x:c r="J89" s="56" t="n">
-        <x:v>97.19728094012108</x:v>
-      </x:c>
+        <x:v>0.5315107139042438</x:v>
+      </x:c>
+      <x:c r="J89" s="56"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="50" t="str">
-        <x:v>8.1</x:v>
+        <x:v>7.2</x:v>
       </x:c>
       <x:c r="B90" s="50" t="str">
-        <x:v>Infusion reaction at 18 months</x:v>
+        <x:v>NPI-Q score at 18 months</x:v>
       </x:c>
       <x:c r="C90" s="50" t="str">
-        <x:v>RR</x:v>
+        <x:v>SMD</x:v>
       </x:c>
       <x:c r="D90" s="50" t="str">
-        <x:v>Exclude futility-terminated trials</x:v>
+        <x:v>Cochrane class pool</x:v>
       </x:c>
       <x:c r="E90" s="59" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="F90" s="62" t="n">
-        <x:v>7.662918735750597</x:v>
+        <x:v>0.1191993997701558</x:v>
       </x:c>
       <x:c r="G90" s="62" t="n">
-        <x:v>1.50871167336935</x:v>
+        <x:v>-0.1747924558477071</x:v>
       </x:c>
       <x:c r="H90" s="62" t="n">
-        <x:v>38.92083861164777</x:v>
+        <x:v>0.4131912553880188</x:v>
       </x:c>
       <x:c r="I90" s="65" t="n">
-        <x:v>0.01405122319592295</x:v>
+        <x:v>0.4268054428964087</x:v>
       </x:c>
       <x:c r="J90" s="56" t="n">
-        <x:v>89.95729838569783</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="50" t="str">
-        <x:v>8.1</x:v>
+        <x:v>7.2</x:v>
       </x:c>
       <x:c r="B91" s="50" t="str">
-        <x:v>Infusion reaction at 18 months</x:v>
+        <x:v>NPI-Q score at 18 months</x:v>
       </x:c>
       <x:c r="C91" s="50" t="str">
-        <x:v>RR</x:v>
+        <x:v>SMD</x:v>
       </x:c>
       <x:c r="D91" s="50" t="str">
-        <x:v>Exclude all early-terminated trials</x:v>
+        <x:v>Exclude futility-terminated trials</x:v>
       </x:c>
       <x:c r="E91" s="59" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F91" s="62" t="n">
-        <x:v>7.662918735750597</x:v>
+        <x:v>0.5168562568898105</x:v>
       </x:c>
       <x:c r="G91" s="62" t="n">
-        <x:v>1.50871167336935</x:v>
+        <x:v>-0.9579855762756353</x:v>
       </x:c>
       <x:c r="H91" s="62" t="n">
-        <x:v>38.92083861164777</x:v>
+        <x:v>1.991698090055256</x:v>
       </x:c>
       <x:c r="I91" s="65" t="n">
-        <x:v>0.01405122319592295</x:v>
-      </x:c>
-      <x:c r="J91" s="56" t="n">
-        <x:v>89.95729838569783</x:v>
-      </x:c>
+        <x:v>0.4921667733628572</x:v>
+      </x:c>
+      <x:c r="J91" s="56"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="50" t="str">
-        <x:v>8.2</x:v>
+        <x:v>8.1</x:v>
       </x:c>
       <x:c r="B92" s="50" t="str">
-        <x:v>Infusion reaction at 24 months</x:v>
+        <x:v>Infusion reaction at 18 months</x:v>
       </x:c>
       <x:c r="C92" s="50" t="str">
         <x:v>RR</x:v>
@@ -14281,124 +14275,124 @@
         <x:v>Cochrane class pool</x:v>
       </x:c>
       <x:c r="E92" s="59" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F92" s="62" t="n">
-        <x:v>1.149178942284472</x:v>
+        <x:v>3.580414000675479</x:v>
       </x:c>
       <x:c r="G92" s="62" t="n">
-        <x:v>0.7737788248778547</x:v>
+        <x:v>0.06906491805724485</x:v>
       </x:c>
       <x:c r="H92" s="62" t="n">
-        <x:v>1.706705067302049</x:v>
+        <x:v>185.61325745159925</x:v>
       </x:c>
       <x:c r="I92" s="65" t="n">
-        <x:v>0.4907956322652618</x:v>
-      </x:c>
-      <x:c r="J92" s="56"/>
+        <x:v>0.2990275366168896</x:v>
+      </x:c>
+      <x:c r="J92" s="56" t="n">
+        <x:v>97.19728094012108</x:v>
+      </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="50" t="str">
-        <x:v>9.1</x:v>
+        <x:v>8.1</x:v>
       </x:c>
       <x:c r="B93" s="50" t="str">
-        <x:v>Study discontinuation at 18 months</x:v>
+        <x:v>Infusion reaction at 18 months</x:v>
       </x:c>
       <x:c r="C93" s="50" t="str">
         <x:v>RR</x:v>
       </x:c>
       <x:c r="D93" s="50" t="str">
-        <x:v>Cochrane class pool</x:v>
+        <x:v>Exclude futility-terminated trials</x:v>
       </x:c>
       <x:c r="E93" s="59" t="n">
-        <x:v>11</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F93" s="62" t="n">
-        <x:v>1.12069436507818</x:v>
+        <x:v>7.662918735750597</x:v>
       </x:c>
       <x:c r="G93" s="62" t="n">
-        <x:v>1.020569085776655</x:v>
+        <x:v>1.50871167336935</x:v>
       </x:c>
       <x:c r="H93" s="62" t="n">
-        <x:v>1.230642665373507</x:v>
+        <x:v>38.92083861164777</x:v>
       </x:c>
       <x:c r="I93" s="65" t="n">
-        <x:v>0.02182552233863456</x:v>
+        <x:v>0.01405122319592295</x:v>
       </x:c>
       <x:c r="J93" s="56" t="n">
-        <x:v>49.554731620791884</x:v>
+        <x:v>89.95729838569783</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="50" t="str">
-        <x:v>9.1</x:v>
+        <x:v>8.1</x:v>
       </x:c>
       <x:c r="B94" s="50" t="str">
-        <x:v>Study discontinuation at 18 months</x:v>
+        <x:v>Infusion reaction at 18 months</x:v>
       </x:c>
       <x:c r="C94" s="50" t="str">
         <x:v>RR</x:v>
       </x:c>
       <x:c r="D94" s="50" t="str">
-        <x:v>Exclude futility-terminated trials</x:v>
+        <x:v>Exclude all early-terminated trials</x:v>
       </x:c>
       <x:c r="E94" s="59" t="n">
-        <x:v>8</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F94" s="62" t="n">
-        <x:v>1.094865043171826</x:v>
+        <x:v>7.662918735750597</x:v>
       </x:c>
       <x:c r="G94" s="62" t="n">
-        <x:v>0.975234787266681</x:v>
+        <x:v>1.50871167336935</x:v>
       </x:c>
       <x:c r="H94" s="62" t="n">
-        <x:v>1.22917012232445</x:v>
+        <x:v>38.92083861164777</x:v>
       </x:c>
       <x:c r="I94" s="65" t="n">
-        <x:v>0.1064311876264151</x:v>
+        <x:v>0.01405122319592295</x:v>
       </x:c>
       <x:c r="J94" s="56" t="n">
-        <x:v>57.71107193589428</x:v>
+        <x:v>89.95729838569783</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="50" t="str">
-        <x:v>9.1</x:v>
+        <x:v>8.2</x:v>
       </x:c>
       <x:c r="B95" s="50" t="str">
-        <x:v>Study discontinuation at 18 months</x:v>
+        <x:v>Infusion reaction at 24 months</x:v>
       </x:c>
       <x:c r="C95" s="50" t="str">
         <x:v>RR</x:v>
       </x:c>
       <x:c r="D95" s="50" t="str">
-        <x:v>Exclude all early-terminated trials</x:v>
+        <x:v>Cochrane class pool</x:v>
       </x:c>
       <x:c r="E95" s="59" t="n">
-        <x:v>6</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F95" s="62" t="n">
-        <x:v>1.123735951757978</x:v>
+        <x:v>1.149178942284472</x:v>
       </x:c>
       <x:c r="G95" s="62" t="n">
-        <x:v>0.9563543981977306</x:v>
+        <x:v>0.7737788248778547</x:v>
       </x:c>
       <x:c r="H95" s="62" t="n">
-        <x:v>1.320412696018493</x:v>
+        <x:v>1.706705067302049</x:v>
       </x:c>
       <x:c r="I95" s="65" t="n">
-        <x:v>0.1220778201885251</x:v>
-      </x:c>
-      <x:c r="J95" s="56" t="n">
-        <x:v>58.930562054410665</x:v>
-      </x:c>
+        <x:v>0.4907956322652618</x:v>
+      </x:c>
+      <x:c r="J95" s="56"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="50" t="str">
-        <x:v>9.2</x:v>
+        <x:v>9.1</x:v>
       </x:c>
       <x:c r="B96" s="50" t="str">
-        <x:v>Study discontinuation at 24 months</x:v>
+        <x:v>Study discontinuation at 18 months</x:v>
       </x:c>
       <x:c r="C96" s="50" t="str">
         <x:v>RR</x:v>
@@ -14407,117 +14401,213 @@
         <x:v>Cochrane class pool</x:v>
       </x:c>
       <x:c r="E96" s="59" t="n">
-        <x:v>2</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F96" s="62" t="n">
-        <x:v>1.008741777821183</x:v>
+        <x:v>1.12069436507818</x:v>
       </x:c>
       <x:c r="G96" s="62" t="n">
-        <x:v>0.9411188324553127</x:v>
+        <x:v>1.020569085776655</x:v>
       </x:c>
       <x:c r="H96" s="62" t="n">
-        <x:v>1.081223687413734</x:v>
+        <x:v>1.230642665373507</x:v>
       </x:c>
       <x:c r="I96" s="65" t="n">
-        <x:v>0.8058020547192903</x:v>
+        <x:v>0.02182552233863456</x:v>
       </x:c>
       <x:c r="J96" s="56" t="n">
-        <x:v>0</x:v>
+        <x:v>49.554731620791884</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="50" t="str">
-        <x:v>9.3</x:v>
+        <x:v>9.1</x:v>
       </x:c>
       <x:c r="B97" s="50" t="str">
-        <x:v>Study discontinuation above 24 months</x:v>
+        <x:v>Study discontinuation at 18 months</x:v>
       </x:c>
       <x:c r="C97" s="50" t="str">
         <x:v>RR</x:v>
       </x:c>
       <x:c r="D97" s="50" t="str">
-        <x:v>Cochrane class pool</x:v>
+        <x:v>Exclude futility-terminated trials</x:v>
       </x:c>
       <x:c r="E97" s="59" t="n">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F97" s="62" t="n">
-        <x:v>1.355002688994968</x:v>
+        <x:v>1.094865043171826</x:v>
       </x:c>
       <x:c r="G97" s="62" t="n">
-        <x:v>1.109422105329669</x:v>
+        <x:v>0.975234787266681</x:v>
       </x:c>
       <x:c r="H97" s="62" t="n">
-        <x:v>1.654944748588734</x:v>
+        <x:v>1.22917012232445</x:v>
       </x:c>
       <x:c r="I97" s="65" t="n">
-        <x:v>0.002903706094042277</x:v>
+        <x:v>0.1064311876264151</x:v>
       </x:c>
       <x:c r="J97" s="56" t="n">
-        <x:v>26.853249664784688</x:v>
+        <x:v>57.71107193589428</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="50" t="str">
-        <x:v>9.3</x:v>
+        <x:v>9.1</x:v>
       </x:c>
       <x:c r="B98" s="50" t="str">
-        <x:v>Study discontinuation above 24 months</x:v>
+        <x:v>Study discontinuation at 18 months</x:v>
       </x:c>
       <x:c r="C98" s="50" t="str">
         <x:v>RR</x:v>
       </x:c>
       <x:c r="D98" s="50" t="str">
+        <x:v>Exclude all early-terminated trials</x:v>
+      </x:c>
+      <x:c r="E98" s="59" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F98" s="62" t="n">
+        <x:v>1.123735951757978</x:v>
+      </x:c>
+      <x:c r="G98" s="62" t="n">
+        <x:v>0.9563543981977306</x:v>
+      </x:c>
+      <x:c r="H98" s="62" t="n">
+        <x:v>1.320412696018493</x:v>
+      </x:c>
+      <x:c r="I98" s="65" t="n">
+        <x:v>0.1220778201885251</x:v>
+      </x:c>
+      <x:c r="J98" s="56" t="n">
+        <x:v>58.930562054410665</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" s="50" t="str">
+        <x:v>9.2</x:v>
+      </x:c>
+      <x:c r="B99" s="50" t="str">
+        <x:v>Study discontinuation at 24 months</x:v>
+      </x:c>
+      <x:c r="C99" s="50" t="str">
+        <x:v>RR</x:v>
+      </x:c>
+      <x:c r="D99" s="50" t="str">
+        <x:v>Cochrane class pool</x:v>
+      </x:c>
+      <x:c r="E99" s="59" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F99" s="62" t="n">
+        <x:v>1.008741777821183</x:v>
+      </x:c>
+      <x:c r="G99" s="62" t="n">
+        <x:v>0.9411188324553127</x:v>
+      </x:c>
+      <x:c r="H99" s="62" t="n">
+        <x:v>1.081223687413734</x:v>
+      </x:c>
+      <x:c r="I99" s="65" t="n">
+        <x:v>0.8058020547192903</x:v>
+      </x:c>
+      <x:c r="J99" s="56" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" s="50" t="str">
+        <x:v>9.3</x:v>
+      </x:c>
+      <x:c r="B100" s="50" t="str">
+        <x:v>Study discontinuation above 24 months</x:v>
+      </x:c>
+      <x:c r="C100" s="50" t="str">
+        <x:v>RR</x:v>
+      </x:c>
+      <x:c r="D100" s="50" t="str">
+        <x:v>Cochrane class pool</x:v>
+      </x:c>
+      <x:c r="E100" s="59" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F100" s="62" t="n">
+        <x:v>1.355002688994968</x:v>
+      </x:c>
+      <x:c r="G100" s="62" t="n">
+        <x:v>1.109422105329669</x:v>
+      </x:c>
+      <x:c r="H100" s="62" t="n">
+        <x:v>1.654944748588734</x:v>
+      </x:c>
+      <x:c r="I100" s="65" t="n">
+        <x:v>0.002903706094042277</x:v>
+      </x:c>
+      <x:c r="J100" s="56" t="n">
+        <x:v>26.853249664784688</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" s="50" t="str">
+        <x:v>9.3</x:v>
+      </x:c>
+      <x:c r="B101" s="50" t="str">
+        <x:v>Study discontinuation above 24 months</x:v>
+      </x:c>
+      <x:c r="C101" s="50" t="str">
+        <x:v>RR</x:v>
+      </x:c>
+      <x:c r="D101" s="50" t="str">
         <x:v>Exclude futility-terminated trials</x:v>
       </x:c>
-      <x:c r="E98" s="59" t="n">
+      <x:c r="E101" s="59" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="F98" s="62" t="n">
+      <x:c r="F101" s="62" t="n">
         <x:v>1.355002688994968</x:v>
       </x:c>
-      <x:c r="G98" s="62" t="n">
+      <x:c r="G101" s="62" t="n">
         <x:v>1.109422105329669</x:v>
       </x:c>
-      <x:c r="H98" s="62" t="n">
+      <x:c r="H101" s="62" t="n">
         <x:v>1.654944748588734</x:v>
       </x:c>
-      <x:c r="I98" s="65" t="n">
+      <x:c r="I101" s="65" t="n">
         <x:v>0.002903706094042277</x:v>
       </x:c>
-      <x:c r="J98" s="56" t="n">
+      <x:c r="J101" s="56" t="n">
         <x:v>26.853249664784688</x:v>
       </x:c>
     </x:row>
-    <x:row r="99">
-      <x:c r="A99" s="51" t="str">
+    <x:row r="102">
+      <x:c r="A102" s="51" t="str">
         <x:v>9.3</x:v>
       </x:c>
-      <x:c r="B99" s="51" t="str">
+      <x:c r="B102" s="51" t="str">
         <x:v>Study discontinuation above 24 months</x:v>
       </x:c>
-      <x:c r="C99" s="51" t="str">
+      <x:c r="C102" s="51" t="str">
         <x:v>RR</x:v>
       </x:c>
-      <x:c r="D99" s="51" t="str">
+      <x:c r="D102" s="51" t="str">
         <x:v>Exclude all early-terminated trials</x:v>
       </x:c>
-      <x:c r="E99" s="60" t="n">
+      <x:c r="E102" s="60" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="F99" s="63" t="n">
+      <x:c r="F102" s="63" t="n">
         <x:v>1.355002688994968</x:v>
       </x:c>
-      <x:c r="G99" s="63" t="n">
+      <x:c r="G102" s="63" t="n">
         <x:v>1.109422105329669</x:v>
       </x:c>
-      <x:c r="H99" s="63" t="n">
+      <x:c r="H102" s="63" t="n">
         <x:v>1.654944748588734</x:v>
       </x:c>
-      <x:c r="I99" s="66" t="n">
+      <x:c r="I102" s="66" t="n">
         <x:v>0.002903706094042277</x:v>
       </x:c>
-      <x:c r="J99" s="57" t="n">
+      <x:c r="J102" s="57" t="n">
         <x:v>26.853249664784688</x:v>
       </x:c>
     </x:row>
@@ -14528,7 +14618,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a6222de622e4df7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf9731a154eb4cde"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15238,7 +15328,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a7675a1ce0542fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebfeaff9d75945b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16404,7 +16494,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07470e1c399048a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R386027031397499b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>